<commit_message>
improve formulas for uncertainty in overall dec vote bias
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4DCD380-6DCB-4789-A946-C7489F8C2A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6959E860-42BD-445B-80FC-E8EE81D49D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16200" yWindow="5565" windowWidth="24345" windowHeight="17730" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="12315" yWindow="5145" windowWidth="25140" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -471,16 +472,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B2">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D2">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -495,29 +496,29 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>A2*100/$K$2</f>
-        <v>24.242424242424242</v>
+        <v>27.083333333333332</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:I4" si="0">B2*100/$K$2</f>
-        <v>35.353535353535356</v>
+        <v>31.25</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>6.0606060606060606</v>
+        <v>11.458333333333334</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>16.161616161616163</v>
+        <v>22.916666666666668</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -537,7 +538,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>18.181818181818183</v>
+        <v>7.291666666666667</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -548,19 +549,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>24.242424242424242</v>
+        <v>27.083333333333332</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>35.353535353535356</v>
+        <v>31.25</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>6.0606060606060606</v>
+        <v>11.458333333333334</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>16.161616161616163</v>
+        <v>22.916666666666668</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -580,7 +581,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>18.181818181818183</v>
+        <v>7.291666666666667</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -619,7 +620,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>54.728686868686879</v>
+        <v>51.172812499999999</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -631,25 +632,25 @@
       </c>
       <c r="D9">
         <f>SUM(A10:B10)</f>
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B10">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <f>A10*100/D9</f>
-        <v>47.872340425531917</v>
+        <v>50.526315789473685</v>
       </c>
       <c r="B11">
         <f>B10*100/D9</f>
-        <v>52.127659574468083</v>
+        <v>49.473684210526315</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
prepare for 2026sa live data ingestion
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6959E860-42BD-445B-80FC-E8EE81D49D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAEC4C48-6CA2-4C2E-9158-94FE37B5EFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12315" yWindow="5145" windowWidth="25140" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="11460" yWindow="4575" windowWidth="28530" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -472,16 +471,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B2">
         <v>30</v>
       </c>
       <c r="C2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -496,29 +495,29 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>A2*100/$K$2</f>
-        <v>27.083333333333332</v>
+        <v>20.202020202020201</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:I4" si="0">B2*100/$K$2</f>
-        <v>31.25</v>
+        <v>30.303030303030305</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>11.458333333333334</v>
+        <v>12.121212121212121</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>22.916666666666668</v>
+        <v>19.19191919191919</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -538,7 +537,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>7.291666666666667</v>
+        <v>18.181818181818183</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -549,19 +548,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>27.083333333333332</v>
+        <v>20.202020202020201</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>31.25</v>
+        <v>30.303030303030305</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>11.458333333333334</v>
+        <v>12.121212121212121</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>22.916666666666668</v>
+        <v>19.19191919191919</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -581,7 +580,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>7.291666666666667</v>
+        <v>18.181818181818183</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -620,7 +619,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>51.172812499999999</v>
+        <v>55.795757575757577</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
initial live booth snapshot screen (internal) + routine update
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAEC4C48-6CA2-4C2E-9158-94FE37B5EFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{381DBE67-DC32-4385-A9B2-A97C55DD1888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11460" yWindow="4575" windowWidth="28530" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="9060" yWindow="3240" windowWidth="25140" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -471,16 +472,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B2">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C2">
         <v>12</v>
       </c>
       <c r="D2">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -495,29 +496,30 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <v>18</v>
+        <f>100-SUM(A2:D2)</f>
+        <v>9</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>A2*100/$K$2</f>
-        <v>20.202020202020201</v>
+        <v>13</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:I4" si="0">B2*100/$K$2</f>
-        <v>30.303030303030305</v>
+        <v>39</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>12.121212121212121</v>
+        <v>12</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>19.19191919191919</v>
+        <v>27</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -537,7 +539,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>18.181818181818183</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -548,19 +550,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>20.202020202020201</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>30.303030303030305</v>
+        <v>39</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>12.121212121212121</v>
+        <v>12</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>19.19191919191919</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -580,7 +582,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>18.181818181818183</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -619,7 +621,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>55.795757575757577</v>
+        <v>61.372799999999998</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update for Farrer by-election
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{381DBE67-DC32-4385-A9B2-A97C55DD1888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EF78028-8821-4C00-8EBA-0611F767590B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9060" yWindow="3240" windowWidth="25140" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="25140" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -472,16 +472,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B2">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -496,30 +496,29 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <f>100-SUM(A2:D2)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>A2*100/$K$2</f>
-        <v>13</v>
+        <v>21.212121212121211</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:I4" si="0">B2*100/$K$2</f>
-        <v>39</v>
+        <v>36.363636363636367</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>14.141414141414142</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>22.222222222222221</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -539,7 +538,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>6.0606060606060606</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -550,19 +549,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>13</v>
+        <v>21.212121212121211</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>39</v>
+        <v>36.363636363636367</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>14.141414141414142</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>27</v>
+        <v>22.222222222222221</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -582,7 +581,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>6.0606060606060606</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -621,7 +620,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>61.372799999999998</v>
+        <v>57.804646464646467</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
make regular generation plan include region trends
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2803304C-0951-4AF2-8346-74D1DF11E9AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C490F73D-06FC-4150-A395-1597B9987468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11370" yWindow="3750" windowWidth="25140" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="435" yWindow="885" windowWidth="29610" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -471,16 +471,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B2">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -495,29 +495,29 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:I4" si="0">A2*100/$K$2</f>
-        <v>22.916666666666668</v>
+        <v>23.762376237623762</v>
       </c>
       <c r="B4">
         <f t="shared" si="0"/>
-        <v>32.291666666666664</v>
+        <v>27.722772277227723</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>12.5</v>
+        <v>13.861386138613861</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>26.041666666666668</v>
+        <v>22.772277227722771</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -537,7 +537,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>6.25</v>
+        <v>11.881188118811881</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -548,19 +548,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>22.916666666666668</v>
+        <v>23.762376237623762</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>32.291666666666664</v>
+        <v>27.722772277227723</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>12.5</v>
+        <v>13.861386138613861</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>26.041666666666668</v>
+        <v>22.772277227722771</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -580,7 +580,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>6.25</v>
+        <v>11.881188118811881</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -619,7 +619,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>53.362291666666664</v>
+        <v>52.22930693069307</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>